<commit_message>
Using the right schedule file this time
</commit_message>
<xml_diff>
--- a/math121-schedule-7-11-2026.xlsx
+++ b/math121-schedule-7-11-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dickinson0-my.sharepoint.com/personal/jmac_dickinson_edu/Documents/repository/courses/ai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="242" documentId="13_ncr:1_{91DEECA4-1339-44A4-B91E-F265F67426BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1C65C9D-48E2-4E16-AB63-DFB3CE95CA5F}"/>
+  <xr:revisionPtr revIDLastSave="315" documentId="13_ncr:1_{91DEECA4-1339-44A4-B91E-F265F67426BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4EAC01F-98B4-4B83-A445-6A6339791687}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t>Class number</t>
   </si>
@@ -41,9 +41,6 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Tue</t>
-  </si>
-  <si>
     <t>topic</t>
   </si>
   <si>
@@ -149,175 +146,64 @@
     <t>thanksgiving vacation</t>
   </si>
   <si>
-    <t>12/18, 2pm-5pm</t>
-  </si>
-  <si>
     <t>exam review</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Convolutional neural networks </t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Reinforcement learning </t>
-  </si>
-  <si>
     <t>Required reading</t>
   </si>
   <si>
-    <t>HW1</t>
-  </si>
-  <si>
-    <t>HW2</t>
-  </si>
-  <si>
-    <t>HW3</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">2. Elementary classifiers: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>nearest neighbor and decision tree</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">3. Neural networks </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>and backpropagation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t>1. Classical search</t>
-  </si>
-  <si>
-    <t>8. Final project</t>
-  </si>
-  <si>
-    <t>ThinkingAI5-7</t>
-  </si>
-  <si>
-    <t>ThinkingAI8-10</t>
-  </si>
-  <si>
-    <t>ThinkingAI1-4 + Turing1950</t>
-  </si>
-  <si>
     <t>homework due + quizzes</t>
   </si>
   <si>
-    <t>Q1</t>
-  </si>
-  <si>
-    <t>Q2</t>
-  </si>
-  <si>
-    <t>Q3</t>
-  </si>
-  <si>
-    <t>ThinkingAI11 + searle1980</t>
-  </si>
-  <si>
-    <t>ThinkingAI12-14</t>
-  </si>
-  <si>
-    <t>[final project]</t>
-  </si>
-  <si>
-    <t>final presentations/posters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Special topic: AI and sustainability </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">SP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(sustainability poster in class)</t>
-    </r>
-  </si>
-  <si>
-    <t>Q4</t>
-  </si>
-  <si>
-    <t>HW4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Transformers and large language models </t>
-  </si>
-  <si>
-    <t>Q6</t>
-  </si>
-  <si>
-    <t>HW6</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Q5
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(no HW5)</t>
-    </r>
-  </si>
-  <si>
-    <t>FP1</t>
-  </si>
-  <si>
-    <t>FP2</t>
-  </si>
-  <si>
-    <t>FP3</t>
+    <t>Mon</t>
+  </si>
+  <si>
+    <t>Thu</t>
+  </si>
+  <si>
+    <t>12/18, 9am-12pm</t>
+  </si>
+  <si>
+    <t>final exam</t>
+  </si>
+  <si>
+    <t>midterm exam 3</t>
+  </si>
+  <si>
+    <t>Topic 10: Confidence Intervals and Hypothesis Tests of Two Proportions</t>
+  </si>
+  <si>
+    <t>[review]</t>
+  </si>
+  <si>
+    <t>Topic 0: How to Make a Decision with Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topic 1: Introduction to Data </t>
+  </si>
+  <si>
+    <t>Topic 2: Picturing Variation with Graphs</t>
+  </si>
+  <si>
+    <t>Topic 3: Numerical Summaries of Center and Variation</t>
+  </si>
+  <si>
+    <t>Topic 4: Regression Analysis: Exploring Associations Between Variables</t>
+  </si>
+  <si>
+    <t>Topic 5: Modeling Variation with Probability</t>
+  </si>
+  <si>
+    <t>Topic 6: Modeling Random Events: The Normal and Uniform Models</t>
+  </si>
+  <si>
+    <t>Topic 7: Survey Sampling and Inference</t>
+  </si>
+  <si>
+    <t>Topic 8: Hypothesis Testing for Population Proportions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topic 9: Inferring Population Means </t>
   </si>
 </sst>
 </file>
@@ -327,7 +213,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,21 +280,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -453,7 +325,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -476,6 +348,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -596,7 +494,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -611,18 +509,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -633,6 +522,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,10 +546,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -950,7 +844,7 @@
     <col min="1" max="1" width="6.140625" style="10" customWidth="1"/>
     <col min="2" max="2" width="5.140625" style="30" customWidth="1"/>
     <col min="3" max="3" width="6.42578125" style="22" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="36" style="8" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" style="10" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" style="10" customWidth="1"/>
     <col min="7" max="7" width="25.28515625" style="22" customWidth="1"/>
@@ -958,9 +852,9 @@
     <col min="9" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="7" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="7" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -968,35 +862,35 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="47" t="s">
-        <v>4</v>
+      <c r="D1" s="46" t="s">
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="33" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H1"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12">
         <v>1</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="C2" s="23">
-        <v>46266</v>
-      </c>
-      <c r="D2" s="48" t="s">
-        <v>49</v>
+        <v>46265</v>
+      </c>
+      <c r="D2" s="52" t="s">
+        <v>48</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" s="36"/>
       <c r="G2" s="18"/>
@@ -1004,15 +898,15 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
       <c r="B3" s="27" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C3" s="23">
         <f>C2+3</f>
-        <v>46269</v>
-      </c>
-      <c r="D3" s="48"/>
+        <v>46268</v>
+      </c>
+      <c r="D3" s="53"/>
       <c r="E3" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3" s="36"/>
       <c r="G3" s="19"/>
@@ -1024,15 +918,17 @@
       </c>
       <c r="B4" s="27" t="str">
         <f>B2</f>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C4" s="23">
         <f>C2+7</f>
-        <v>46273</v>
-      </c>
-      <c r="D4" s="48"/>
+        <v>46272</v>
+      </c>
+      <c r="D4" s="51" t="s">
+        <v>49</v>
+      </c>
       <c r="E4" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4" s="36"/>
       <c r="G4" s="18"/>
@@ -1041,21 +937,19 @@
       <c r="A5" s="12"/>
       <c r="B5" s="27" t="str">
         <f>B3</f>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C5" s="23">
         <f>C3+7</f>
-        <v>46276</v>
-      </c>
-      <c r="D5" s="48" t="s">
-        <v>47</v>
+        <v>46275</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>50</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="36" t="s">
-        <v>55</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F5" s="36"/>
       <c r="G5" s="19"/>
     </row>
     <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1065,36 +959,34 @@
       </c>
       <c r="B6" s="27" t="str">
         <f t="shared" ref="B6:B31" si="1">B4</f>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C6" s="23">
         <f t="shared" ref="C6:C31" si="2">C4+7</f>
-        <v>46280</v>
-      </c>
-      <c r="D6" s="48"/>
+        <v>46279</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>51</v>
+      </c>
       <c r="E6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>44</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="F6" s="36"/>
       <c r="G6" s="19"/>
     </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12"/>
       <c r="B7" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C7" s="23">
         <f t="shared" si="2"/>
-        <v>46283</v>
-      </c>
-      <c r="D7" s="49" t="s">
-        <v>53</v>
-      </c>
+        <v>46282</v>
+      </c>
+      <c r="D7" s="53"/>
       <c r="E7" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" s="36"/>
       <c r="G7" s="18"/>
@@ -1106,40 +998,36 @@
       </c>
       <c r="B8" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C8" s="23">
         <f t="shared" si="2"/>
-        <v>46287</v>
-      </c>
-      <c r="D8" s="48" t="s">
-        <v>48</v>
+        <v>46286</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>52</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="36" t="s">
-        <v>56</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F8" s="36"/>
       <c r="G8" s="34"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="12"/>
       <c r="B9" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C9" s="23">
         <f t="shared" si="2"/>
-        <v>46290</v>
-      </c>
-      <c r="D9" s="48"/>
+        <v>46289</v>
+      </c>
+      <c r="D9" s="53"/>
       <c r="E9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="36" t="s">
-        <v>45</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="F9" s="36"/>
       <c r="G9" s="35"/>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1149,17 +1037,17 @@
       </c>
       <c r="B10" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C10" s="23">
         <f t="shared" si="2"/>
-        <v>46294</v>
-      </c>
-      <c r="D10" s="48" t="s">
-        <v>62</v>
+        <v>46293</v>
+      </c>
+      <c r="D10" s="47" t="s">
+        <v>38</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G10" s="35"/>
     </row>
@@ -1167,19 +1055,19 @@
       <c r="A11" s="12"/>
       <c r="B11" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C11" s="23">
         <f t="shared" si="2"/>
-        <v>46297</v>
-      </c>
-      <c r="D11" s="48"/>
+        <v>46296</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>33</v>
+      </c>
       <c r="E11" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" s="36" t="s">
-        <v>57</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="F11" s="36"/>
       <c r="G11" s="35"/>
     </row>
     <row r="12" spans="1:8" s="15" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1189,19 +1077,19 @@
       </c>
       <c r="B12" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C12" s="24">
         <f t="shared" si="2"/>
-        <v>46301</v>
-      </c>
-      <c r="D12" s="48"/>
+        <v>46300</v>
+      </c>
+      <c r="D12" s="52" t="s">
+        <v>53</v>
+      </c>
       <c r="E12" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="44" t="s">
-        <v>63</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="F12" s="44"/>
       <c r="G12" s="20"/>
       <c r="H12"/>
     </row>
@@ -1209,41 +1097,37 @@
       <c r="A13" s="12"/>
       <c r="B13" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C13" s="23">
         <f t="shared" si="2"/>
-        <v>46304</v>
-      </c>
-      <c r="D13" s="50" t="s">
-        <v>40</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="D13" s="53"/>
       <c r="E13" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>46</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F13" s="36"/>
       <c r="G13" s="18"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <f t="shared" ref="A14" si="6">A12+1</f>
         <v>7</v>
       </c>
       <c r="B14" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C14" s="23">
         <f t="shared" si="2"/>
-        <v>46308</v>
-      </c>
-      <c r="D14" s="51" t="s">
-        <v>34</v>
+        <v>46307</v>
+      </c>
+      <c r="D14" s="52" t="s">
+        <v>54</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F14" s="36"/>
       <c r="G14" s="19"/>
@@ -1252,17 +1136,15 @@
       <c r="A15" s="12"/>
       <c r="B15" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C15" s="23">
         <f t="shared" si="2"/>
-        <v>46311</v>
-      </c>
-      <c r="D15" s="49" t="s">
-        <v>51</v>
-      </c>
+        <v>46310</v>
+      </c>
+      <c r="D15" s="53"/>
       <c r="E15" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F15" s="36"/>
       <c r="G15" s="18"/>
@@ -1271,14 +1153,14 @@
       <c r="A16" s="12"/>
       <c r="B16" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C16" s="23">
         <f t="shared" si="2"/>
-        <v>46315</v>
-      </c>
-      <c r="D16" s="52" t="s">
-        <v>37</v>
+        <v>46314</v>
+      </c>
+      <c r="D16" s="49" t="s">
+        <v>36</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="38"/>
@@ -1290,17 +1172,17 @@
       </c>
       <c r="B17" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C17" s="23">
         <f t="shared" si="2"/>
-        <v>46318</v>
-      </c>
-      <c r="D17" s="48" t="s">
-        <v>41</v>
+        <v>46317</v>
+      </c>
+      <c r="D17" s="52" t="s">
+        <v>55</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F17" s="36"/>
       <c r="G17" s="19"/>
@@ -1309,15 +1191,15 @@
       <c r="A18" s="12"/>
       <c r="B18" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C18" s="23">
         <f t="shared" si="2"/>
-        <v>46322</v>
-      </c>
-      <c r="D18" s="48"/>
+        <v>46321</v>
+      </c>
+      <c r="D18" s="53"/>
       <c r="E18" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F18" s="36"/>
       <c r="G18" s="19"/>
@@ -1329,15 +1211,17 @@
       </c>
       <c r="B19" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C19" s="23">
         <f t="shared" si="2"/>
-        <v>46325</v>
-      </c>
-      <c r="D19" s="48"/>
+        <v>46324</v>
+      </c>
+      <c r="D19" s="47" t="s">
+        <v>38</v>
+      </c>
       <c r="E19" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="19"/>
@@ -1346,164 +1230,150 @@
       <c r="A20" s="12"/>
       <c r="B20" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C20" s="23">
         <f t="shared" si="2"/>
-        <v>46329</v>
-      </c>
-      <c r="D20" s="49" t="s">
-        <v>52</v>
+        <v>46328</v>
+      </c>
+      <c r="D20" s="48" t="s">
+        <v>34</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F20" s="45"/>
       <c r="G20" s="19"/>
     </row>
-    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
         <f t="shared" ref="A21" si="7">A19+1</f>
         <v>10</v>
       </c>
       <c r="B21" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C21" s="23">
         <f t="shared" si="2"/>
-        <v>46332</v>
-      </c>
-      <c r="D21" s="46" t="s">
-        <v>42</v>
+        <v>46331</v>
+      </c>
+      <c r="D21" s="52" t="s">
+        <v>56</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>64</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F21" s="12"/>
       <c r="G21" s="26"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
       <c r="B22" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C22" s="23">
         <f t="shared" si="2"/>
-        <v>46336</v>
-      </c>
-      <c r="D22" s="48" t="s">
-        <v>66</v>
-      </c>
+        <v>46335</v>
+      </c>
+      <c r="D22" s="53"/>
       <c r="E22" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>65</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F22" s="12"/>
       <c r="G22" s="19"/>
     </row>
-    <row r="23" spans="1:8" ht="27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
         <f t="shared" ref="A23" si="8">A21+1</f>
         <v>11</v>
       </c>
       <c r="B23" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C23" s="23">
         <f t="shared" si="2"/>
-        <v>46339</v>
-      </c>
-      <c r="D23" s="48"/>
+        <v>46338</v>
+      </c>
+      <c r="D23" s="52" t="s">
+        <v>57</v>
+      </c>
       <c r="E23" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>69</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="F23" s="39"/>
       <c r="G23" s="26"/>
     </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C24" s="23">
         <f t="shared" si="2"/>
-        <v>46343</v>
-      </c>
-      <c r="D24" s="49" t="s">
-        <v>58</v>
-      </c>
+        <v>46342</v>
+      </c>
+      <c r="D24" s="53"/>
       <c r="E24" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F24" s="39"/>
       <c r="G24" s="26"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12">
         <f t="shared" ref="A25" si="9">A23+1</f>
         <v>12</v>
       </c>
       <c r="B25" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C25" s="23">
         <f t="shared" si="2"/>
-        <v>46346</v>
-      </c>
-      <c r="D25" s="46" t="s">
-        <v>50</v>
+        <v>46345</v>
+      </c>
+      <c r="D25" s="52" t="s">
+        <v>46</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>67</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="F25" s="12"/>
       <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C26" s="23">
         <f t="shared" si="2"/>
-        <v>46350</v>
-      </c>
-      <c r="D26" s="50" t="s">
-        <v>40</v>
-      </c>
+        <v>46349</v>
+      </c>
+      <c r="D26" s="53"/>
       <c r="E26" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>68</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="F26" s="12"/>
       <c r="G26" s="19"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
       <c r="B27" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C27" s="23">
         <f t="shared" si="2"/>
-        <v>46353</v>
-      </c>
-      <c r="D27" s="52" t="s">
-        <v>38</v>
+        <v>46352</v>
+      </c>
+      <c r="D27" s="49" t="s">
+        <v>37</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="12"/>
@@ -1516,17 +1386,17 @@
       </c>
       <c r="B28" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C28" s="23">
         <f t="shared" si="2"/>
-        <v>46357</v>
-      </c>
-      <c r="D28" s="51" t="s">
-        <v>35</v>
+        <v>46356</v>
+      </c>
+      <c r="D28" s="47" t="s">
+        <v>38</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F28" s="36"/>
       <c r="G28" s="42"/>
@@ -1535,21 +1405,19 @@
       <c r="A29" s="32"/>
       <c r="B29" s="29" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C29" s="25">
         <f t="shared" si="2"/>
-        <v>46360</v>
-      </c>
-      <c r="D29" s="46" t="s">
-        <v>60</v>
+        <v>46359</v>
+      </c>
+      <c r="D29" s="48" t="s">
+        <v>45</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="F29" s="43" t="s">
-        <v>70</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="F29" s="43"/>
       <c r="G29" s="42"/>
       <c r="H29"/>
     </row>
@@ -1560,17 +1428,17 @@
       </c>
       <c r="B30" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C30" s="23">
         <f t="shared" si="2"/>
-        <v>46364</v>
-      </c>
-      <c r="D30" s="49" t="s">
-        <v>59</v>
+        <v>46363</v>
+      </c>
+      <c r="D30" s="52" t="s">
+        <v>47</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F30" s="40"/>
       <c r="G30" s="42"/>
@@ -1579,38 +1447,32 @@
       <c r="A31" s="12"/>
       <c r="B31" s="27" t="str">
         <f t="shared" si="1"/>
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C31" s="23">
         <f t="shared" si="2"/>
-        <v>46367</v>
-      </c>
-      <c r="D31" s="46" t="s">
-        <v>60</v>
-      </c>
+        <v>46366</v>
+      </c>
+      <c r="D31" s="53"/>
       <c r="E31" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F31" s="37" t="s">
-        <v>71</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="F31" s="37"/>
       <c r="G31" s="19"/>
     </row>
     <row r="32" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A32" s="12"/>
       <c r="B32" s="27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C32" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" s="51" t="s">
-        <v>61</v>
+        <v>43</v>
+      </c>
+      <c r="D32" s="48" t="s">
+        <v>44</v>
       </c>
       <c r="E32" s="6"/>
-      <c r="F32" s="36" t="s">
-        <v>72</v>
-      </c>
+      <c r="F32" s="36"/>
       <c r="G32" s="18"/>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.25">
@@ -1618,16 +1480,20 @@
       <c r="G33" s="13"/>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D35" s="53"/>
+      <c r="D35" s="50"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="D5:D6"/>
+  <mergeCells count="10">
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D30:D31"/>
     <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="D23:D24"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished initial draft of schedule and syllabus
</commit_message>
<xml_diff>
--- a/math121-schedule-7-11-2026.xlsx
+++ b/math121-schedule-7-11-2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dickinson0-my.sharepoint.com/personal/jmac_dickinson_edu/Documents/repository/courses/ai/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\math121-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="315" documentId="13_ncr:1_{91DEECA4-1339-44A4-B91E-F265F67426BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4EAC01F-98B4-4B83-A445-6A6339791687}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86188C13-119C-4164-B75A-21DD3B40F2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
   <si>
     <t>Class number</t>
   </si>
@@ -204,6 +204,69 @@
   </si>
   <si>
     <t xml:space="preserve">Topic 9: Inferring Population Means </t>
+  </si>
+  <si>
+    <t>HW0</t>
+  </si>
+  <si>
+    <t>HW1+2</t>
+  </si>
+  <si>
+    <t>HW3</t>
+  </si>
+  <si>
+    <t>HW4</t>
+  </si>
+  <si>
+    <t>HW5</t>
+  </si>
+  <si>
+    <t>HW6</t>
+  </si>
+  <si>
+    <t>HW7</t>
+  </si>
+  <si>
+    <t>HW8</t>
+  </si>
+  <si>
+    <t>HW9</t>
+  </si>
+  <si>
+    <t>HW10</t>
+  </si>
+  <si>
+    <t>ch0</t>
+  </si>
+  <si>
+    <t>ch1</t>
+  </si>
+  <si>
+    <t>ch2</t>
+  </si>
+  <si>
+    <t>ch3</t>
+  </si>
+  <si>
+    <t>ch4</t>
+  </si>
+  <si>
+    <t>ch5</t>
+  </si>
+  <si>
+    <t>ch6</t>
+  </si>
+  <si>
+    <t>ch7</t>
+  </si>
+  <si>
+    <t>ch8</t>
+  </si>
+  <si>
+    <t>ch9</t>
+  </si>
+  <si>
+    <t>ch10</t>
   </si>
 </sst>
 </file>
@@ -287,7 +350,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -303,12 +366,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -378,7 +435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -473,9 +530,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -503,9 +557,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -515,10 +566,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -847,7 +898,7 @@
     <col min="4" max="4" width="36" style="8" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" style="10" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" style="10" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" style="22" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" style="22" customWidth="1"/>
     <col min="8" max="8" width="37.85546875" customWidth="1"/>
     <col min="9" max="16384" width="9.140625" style="9"/>
   </cols>
@@ -862,7 +913,7 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="44" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -886,13 +937,13 @@
       <c r="C2" s="23">
         <v>46265</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="50" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="36"/>
+      <c r="F2" s="35"/>
       <c r="G2" s="18"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -904,12 +955,14 @@
         <f>C2+3</f>
         <v>46268</v>
       </c>
-      <c r="D3" s="53"/>
+      <c r="D3" s="51"/>
       <c r="E3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="36"/>
-      <c r="G3" s="19"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
@@ -924,14 +977,18 @@
         <f>C2+7</f>
         <v>46272</v>
       </c>
-      <c r="D4" s="51" t="s">
+      <c r="D4" s="49" t="s">
         <v>49</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="36"/>
-      <c r="G4" s="18"/>
+      <c r="F4" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12"/>
@@ -943,14 +1000,16 @@
         <f>C3+7</f>
         <v>46275</v>
       </c>
-      <c r="D5" s="51" t="s">
+      <c r="D5" s="49" t="s">
         <v>50</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="36"/>
-      <c r="G5" s="19"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="19" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
@@ -965,14 +1024,18 @@
         <f t="shared" ref="C6:C31" si="2">C4+7</f>
         <v>46279</v>
       </c>
-      <c r="D6" s="52" t="s">
+      <c r="D6" s="50" t="s">
         <v>51</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="36"/>
-      <c r="G6" s="19"/>
+      <c r="F6" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12"/>
@@ -984,11 +1047,11 @@
         <f t="shared" si="2"/>
         <v>46282</v>
       </c>
-      <c r="D7" s="53"/>
+      <c r="D7" s="51"/>
       <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="36"/>
+      <c r="F7" s="35"/>
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1004,14 +1067,18 @@
         <f t="shared" si="2"/>
         <v>46286</v>
       </c>
-      <c r="D8" s="52" t="s">
+      <c r="D8" s="50" t="s">
         <v>52</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="36"/>
-      <c r="G8" s="34"/>
+      <c r="F8" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="12"/>
@@ -1023,12 +1090,12 @@
         <f t="shared" si="2"/>
         <v>46289</v>
       </c>
-      <c r="D9" s="53"/>
+      <c r="D9" s="51"/>
       <c r="E9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="36"/>
-      <c r="G9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="34"/>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
@@ -1043,13 +1110,16 @@
         <f t="shared" si="2"/>
         <v>46293</v>
       </c>
-      <c r="D10" s="47" t="s">
+      <c r="D10" s="45" t="s">
         <v>38</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="35"/>
+      <c r="F10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="34"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
@@ -1061,14 +1131,14 @@
         <f t="shared" si="2"/>
         <v>46296</v>
       </c>
-      <c r="D11" s="48" t="s">
+      <c r="D11" s="46" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="36"/>
-      <c r="G11" s="35"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="34"/>
     </row>
     <row r="12" spans="1:8" s="15" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="31">
@@ -1083,14 +1153,16 @@
         <f t="shared" si="2"/>
         <v>46300</v>
       </c>
-      <c r="D12" s="52" t="s">
+      <c r="D12" s="50" t="s">
         <v>53</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="44"/>
-      <c r="G12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20" t="s">
+        <v>73</v>
+      </c>
       <c r="H12"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,11 +1175,11 @@
         <f t="shared" si="2"/>
         <v>46303</v>
       </c>
-      <c r="D13" s="53"/>
+      <c r="D13" s="51"/>
       <c r="E13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="36"/>
+      <c r="F13" s="35"/>
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1123,14 +1195,18 @@
         <f t="shared" si="2"/>
         <v>46307</v>
       </c>
-      <c r="D14" s="52" t="s">
+      <c r="D14" s="50" t="s">
         <v>54</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="36"/>
-      <c r="G14" s="19"/>
+      <c r="F14" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
@@ -1142,11 +1218,11 @@
         <f t="shared" si="2"/>
         <v>46310</v>
       </c>
-      <c r="D15" s="53"/>
+      <c r="D15" s="51"/>
       <c r="E15" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="36"/>
+      <c r="F15" s="35"/>
       <c r="G15" s="18"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1159,11 +1235,11 @@
         <f t="shared" si="2"/>
         <v>46314</v>
       </c>
-      <c r="D16" s="49" t="s">
+      <c r="D16" s="47" t="s">
         <v>36</v>
       </c>
       <c r="E16" s="11"/>
-      <c r="F16" s="38"/>
+      <c r="F16" s="37"/>
       <c r="G16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1178,14 +1254,18 @@
         <f t="shared" si="2"/>
         <v>46317</v>
       </c>
-      <c r="D17" s="52" t="s">
+      <c r="D17" s="50" t="s">
         <v>55</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="36"/>
-      <c r="G17" s="19"/>
+      <c r="F17" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
@@ -1197,11 +1277,11 @@
         <f t="shared" si="2"/>
         <v>46321</v>
       </c>
-      <c r="D18" s="53"/>
+      <c r="D18" s="51"/>
       <c r="E18" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="36"/>
+      <c r="F18" s="35"/>
       <c r="G18" s="19"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1217,13 +1297,15 @@
         <f t="shared" si="2"/>
         <v>46324</v>
       </c>
-      <c r="D19" s="47" t="s">
+      <c r="D19" s="45" t="s">
         <v>38</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="12"/>
+      <c r="F19" s="12" t="s">
+        <v>64</v>
+      </c>
       <c r="G19" s="19"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1236,13 +1318,13 @@
         <f t="shared" si="2"/>
         <v>46328</v>
       </c>
-      <c r="D20" s="48" t="s">
+      <c r="D20" s="46" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F20" s="45"/>
+      <c r="F20" s="43"/>
       <c r="G20" s="19"/>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1258,14 +1340,16 @@
         <f t="shared" si="2"/>
         <v>46331</v>
       </c>
-      <c r="D21" s="52" t="s">
+      <c r="D21" s="50" t="s">
         <v>56</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>22</v>
       </c>
       <c r="F21" s="12"/>
-      <c r="G21" s="26"/>
+      <c r="G21" s="26" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
@@ -1277,7 +1361,7 @@
         <f t="shared" si="2"/>
         <v>46335</v>
       </c>
-      <c r="D22" s="53"/>
+      <c r="D22" s="51"/>
       <c r="E22" s="6" t="s">
         <v>23</v>
       </c>
@@ -1297,14 +1381,18 @@
         <f t="shared" si="2"/>
         <v>46338</v>
       </c>
-      <c r="D23" s="52" t="s">
+      <c r="D23" s="50" t="s">
         <v>57</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F23" s="39"/>
-      <c r="G23" s="26"/>
+      <c r="F23" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="G23" s="26" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
@@ -1316,11 +1404,11 @@
         <f t="shared" si="2"/>
         <v>46342</v>
       </c>
-      <c r="D24" s="53"/>
+      <c r="D24" s="51"/>
       <c r="E24" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F24" s="39"/>
+      <c r="F24" s="38"/>
       <c r="G24" s="26"/>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1336,14 +1424,18 @@
         <f t="shared" si="2"/>
         <v>46345</v>
       </c>
-      <c r="D25" s="52" t="s">
+      <c r="D25" s="50" t="s">
         <v>46</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F25" s="12"/>
-      <c r="G25" s="19"/>
+      <c r="F25" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
@@ -1355,7 +1447,7 @@
         <f t="shared" si="2"/>
         <v>46349</v>
       </c>
-      <c r="D26" s="53"/>
+      <c r="D26" s="51"/>
       <c r="E26" s="6" t="s">
         <v>27</v>
       </c>
@@ -1372,7 +1464,7 @@
         <f t="shared" si="2"/>
         <v>46352</v>
       </c>
-      <c r="D27" s="49" t="s">
+      <c r="D27" s="47" t="s">
         <v>37</v>
       </c>
       <c r="E27" s="11"/>
@@ -1392,14 +1484,14 @@
         <f t="shared" si="2"/>
         <v>46356</v>
       </c>
-      <c r="D28" s="47" t="s">
+      <c r="D28" s="45" t="s">
         <v>38</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F28" s="36"/>
-      <c r="G28" s="42"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="41"/>
     </row>
     <row r="29" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="32"/>
@@ -1411,14 +1503,14 @@
         <f t="shared" si="2"/>
         <v>46359</v>
       </c>
-      <c r="D29" s="48" t="s">
+      <c r="D29" s="46" t="s">
         <v>45</v>
       </c>
       <c r="E29" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="F29" s="43"/>
-      <c r="G29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="41"/>
       <c r="H29"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1434,14 +1526,16 @@
         <f t="shared" si="2"/>
         <v>46363</v>
       </c>
-      <c r="D30" s="52" t="s">
+      <c r="D30" s="50" t="s">
         <v>47</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F30" s="40"/>
-      <c r="G30" s="42"/>
+      <c r="F30" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="G30" s="41"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
@@ -1453,11 +1547,11 @@
         <f t="shared" si="2"/>
         <v>46366</v>
       </c>
-      <c r="D31" s="53"/>
+      <c r="D31" s="51"/>
       <c r="E31" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F31" s="37"/>
+      <c r="F31" s="36"/>
       <c r="G31" s="19"/>
     </row>
     <row r="32" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
@@ -1465,14 +1559,14 @@
       <c r="B32" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="41" t="s">
+      <c r="C32" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="D32" s="48" t="s">
+      <c r="D32" s="46" t="s">
         <v>44</v>
       </c>
       <c r="E32" s="6"/>
-      <c r="F32" s="36"/>
+      <c r="F32" s="35"/>
       <c r="G32" s="18"/>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.25">
@@ -1480,7 +1574,7 @@
       <c r="G33" s="13"/>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D35" s="50"/>
+      <c r="D35" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>